<commit_message>
data: hourly update 2026-07-15 07:21Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-15.xlsx
+++ b/data/output/workbook/2026-07-15.xlsx
@@ -365,7 +365,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12306300"/>
+    <ext cx="10125075" cy="12877800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 00:10</t>
+          <t>2026-07-15 03:21</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -959,359 +959,123 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="29" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
         <is>
           <t>Los Angeles Sparks offense vs Minnesota Lynx defense</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="30" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B78" s="30" t="inlineStr">
+      <c r="B82" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C78" s="30" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D78" s="30" t="inlineStr">
+      <c r="D82" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E78" s="30" t="inlineStr">
+      <c r="E82" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F78" s="30" t="inlineStr">
+      <c r="F82" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G78" s="30" t="inlineStr">
+      <c r="G82" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H78" s="30" t="inlineStr">
+      <c r="H82" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I78" s="30" t="inlineStr">
+      <c r="I82" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J78" s="30" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K78" s="30" t="inlineStr">
+      <c r="K82" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L78" s="30" t="inlineStr">
+      <c r="L82" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M78" s="30" t="inlineStr">
+      <c r="M82" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N78" s="30" t="inlineStr">
+      <c r="N82" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O78" s="30" t="inlineStr">
+      <c r="O82" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P78" s="30" t="inlineStr">
+      <c r="P82" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q78" s="30" t="inlineStr">
+      <c r="Q82" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="31" t="inlineStr">
-        <is>
-          <t>PPG</t>
-        </is>
-      </c>
-      <c r="B79" s="32" t="n">
-        <v>87.59999999999999</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>87.333</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>85.09999999999999</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>86</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>87.59999999999999</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>88</v>
-      </c>
-      <c r="H79" s="36" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>72.75</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>80</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>78.72199999999999</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>79</v>
-      </c>
-      <c r="P79" s="32" t="n">
-        <v>79.75</v>
-      </c>
-      <c r="Q79" s="34" t="inlineStr">
-        <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B80" s="32" t="n">
-        <v>104.643</v>
-      </c>
-      <c r="C80" s="32" t="n">
-        <v>104.822</v>
-      </c>
-      <c r="D80" s="32" t="n">
-        <v>102.383</v>
-      </c>
-      <c r="E80" s="32" t="n">
-        <v>103.459</v>
-      </c>
-      <c r="F80" s="32" t="n">
-        <v>104.643</v>
-      </c>
-      <c r="G80" s="32" t="n">
-        <v>105.519</v>
-      </c>
-      <c r="H80" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I80" s="32" t="inlineStr"/>
-      <c r="J80" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K80" s="32" t="n">
-        <v>88.01600000000001</v>
-      </c>
-      <c r="L80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="M80" s="32" t="n">
-        <v>97.129</v>
-      </c>
-      <c r="N80" s="32" t="n">
-        <v>96.706</v>
-      </c>
-      <c r="O80" s="32" t="n">
-        <v>98.628</v>
-      </c>
-      <c r="P80" s="32" t="n">
-        <v>95.66500000000001</v>
-      </c>
-      <c r="Q80" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B81" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="C81" s="32" t="n">
-        <v>0.525</v>
-      </c>
-      <c r="D81" s="32" t="n">
-        <v>0.515</v>
-      </c>
-      <c r="E81" s="32" t="n">
-        <v>0.512</v>
-      </c>
-      <c r="F81" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="G81" s="32" t="n">
-        <v>0.525</v>
-      </c>
-      <c r="H81" s="36" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="L81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="M81" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="N81" s="32" t="n">
-        <v>0.464</v>
-      </c>
-      <c r="O81" s="32" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="P81" s="32" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="Q81" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="C82" s="32" t="n">
-        <v>0.546</v>
-      </c>
-      <c r="D82" s="32" t="n">
-        <v>0.546</v>
-      </c>
-      <c r="E82" s="32" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="F82" s="32" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="G82" s="32" t="n">
-        <v>0.498</v>
-      </c>
-      <c r="H82" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="M82" s="32" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="N82" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="O82" s="32" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>0.449</v>
-      </c>
-      <c r="Q82" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>0.328</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>0.321</v>
+        <v>87.333</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>0.302</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>0.303</v>
+        <v>86</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>0.328</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>0.366</v>
+        <v>88</v>
       </c>
       <c r="H83" s="36" t="inlineStr">
         <is>
@@ -1321,127 +1085,115 @@
       <c r="I83" s="32" t="inlineStr"/>
       <c r="J83" s="36" t="inlineStr">
         <is>
-          <t>3rd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="K83" s="32" t="n">
-        <v>0.275</v>
+        <v>72.75</v>
       </c>
       <c r="L83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="M83" s="32" t="n">
-        <v>0.308</v>
+        <v>80</v>
       </c>
       <c r="N83" s="32" t="n">
-        <v>0.311</v>
+        <v>78.72199999999999</v>
       </c>
       <c r="O83" s="32" t="n">
-        <v>0.342</v>
+        <v>79</v>
       </c>
       <c r="P83" s="32" t="n">
-        <v>0.281</v>
+        <v>79.75</v>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.788</v>
+        <v>104.643</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.798</v>
+        <v>104.822</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.79</v>
+        <v>102.383</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.784</v>
+        <v>103.459</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.788</v>
+        <v>104.643</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.8149999999999999</v>
+        <v>105.519</v>
       </c>
       <c r="H84" s="35" t="inlineStr">
         <is>
-          <t>6th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P84" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J84" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="n">
+        <v>88.01600000000001</v>
+      </c>
+      <c r="L84" s="32" t="n">
+        <v>95.66500000000001</v>
+      </c>
+      <c r="M84" s="32" t="n">
+        <v>97.129</v>
+      </c>
+      <c r="N84" s="32" t="n">
+        <v>96.706</v>
+      </c>
+      <c r="O84" s="32" t="n">
+        <v>98.628</v>
+      </c>
+      <c r="P84" s="32" t="n">
+        <v>95.66500000000001</v>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>83.804</v>
+        <v>0.533</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>83.425</v>
+        <v>0.525</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>83.218</v>
+        <v>0.515</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>83.26900000000001</v>
+        <v>0.512</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>83.804</v>
+        <v>0.533</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>83.184</v>
+        <v>0.525</v>
       </c>
       <c r="H85" s="36" t="inlineStr">
         <is>
@@ -1449,275 +1201,251 @@
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P85" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J85" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="L85" s="32" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="M85" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="N85" s="32" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="O85" s="32" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="P85" s="32" t="n">
+        <v>0.441</v>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.584</v>
+        <v>0.544</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.569</v>
+        <v>0.546</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.546</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.538</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.584</v>
+        <v>0.544</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.581</v>
-      </c>
-      <c r="H86" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
+        <v>0.498</v>
+      </c>
+      <c r="H86" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I86" s="32" t="inlineStr"/>
-      <c r="J86" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P86" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J86" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="L86" s="32" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="M86" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="N86" s="32" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="O86" s="32" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="P86" s="32" t="n">
+        <v>0.449</v>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.245</v>
+        <v>0.328</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.237</v>
+        <v>0.321</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.224</v>
+        <v>0.302</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.229</v>
+        <v>0.303</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.245</v>
+        <v>0.328</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="H87" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.366</v>
+      </c>
+      <c r="H87" s="36" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J87" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L87" s="32" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="M87" s="32" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="N87" s="32" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="O87" s="32" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="P87" s="32" t="n">
+        <v>0.281</v>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>29.4</v>
+        <v>0.788</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>32.3</v>
+        <v>0.798</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>31.95</v>
+        <v>0.79</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>30.933</v>
+        <v>0.784</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>29.4</v>
+        <v>0.788</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="H88" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="H88" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="I88" s="32" t="inlineStr"/>
-      <c r="J88" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K88" s="32" t="n">
-        <v>30</v>
-      </c>
-      <c r="L88" s="32" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="M88" s="32" t="n">
-        <v>33.615</v>
-      </c>
-      <c r="N88" s="32" t="n">
-        <v>33.444</v>
-      </c>
-      <c r="O88" s="32" t="n">
-        <v>32.893</v>
-      </c>
-      <c r="P88" s="32" t="n">
-        <v>32.75</v>
+      <c r="J88" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P88" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>19.9</v>
+        <v>83.804</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>20.667</v>
+        <v>83.425</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>19.95</v>
+        <v>83.218</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>20.067</v>
+        <v>83.26900000000001</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>19.9</v>
+        <v>83.804</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="H89" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>83.184</v>
+      </c>
+      <c r="H89" s="36" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -1758,37 +1486,37 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>10.9</v>
+        <v>0.584</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>10.2</v>
+        <v>0.569</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>10.45</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>10.733</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>10.9</v>
+        <v>0.584</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="H90" s="33" t="inlineStr">
-        <is>
-          <t>10th</t>
+        <v>0.581</v>
+      </c>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
@@ -1829,37 +1557,37 @@
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B91" s="32" t="n">
-        <v>16.2</v>
+        <v>0.245</v>
       </c>
       <c r="C91" s="32" t="n">
-        <v>14.233</v>
+        <v>0.237</v>
       </c>
       <c r="D91" s="32" t="n">
-        <v>14.7</v>
+        <v>0.224</v>
       </c>
       <c r="E91" s="32" t="n">
-        <v>14.067</v>
+        <v>0.229</v>
       </c>
       <c r="F91" s="32" t="n">
-        <v>16.2</v>
+        <v>0.245</v>
       </c>
       <c r="G91" s="32" t="n">
-        <v>15</v>
+        <v>0.23</v>
       </c>
       <c r="H91" s="33" t="inlineStr">
         <is>
-          <t>10th</t>
+          <t>11th</t>
         </is>
       </c>
       <c r="I91" s="32" t="inlineStr"/>
@@ -1900,793 +1628,789 @@
       </c>
       <c r="Q91" s="34" t="inlineStr">
         <is>
-          <t>Opp TOV</t>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B92" s="32" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="C92" s="32" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="D92" s="32" t="n">
+        <v>31.95</v>
+      </c>
+      <c r="E92" s="32" t="n">
+        <v>30.933</v>
+      </c>
+      <c r="F92" s="32" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="G92" s="32" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H92" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I92" s="32" t="inlineStr"/>
+      <c r="J92" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K92" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="L92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="M92" s="32" t="n">
+        <v>33.615</v>
+      </c>
+      <c r="N92" s="32" t="n">
+        <v>33.444</v>
+      </c>
+      <c r="O92" s="32" t="n">
+        <v>32.893</v>
+      </c>
+      <c r="P92" s="32" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="Q92" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="inlineStr">
-        <is>
-          <t>Minnesota Lynx offense vs Los Angeles Sparks defense</t>
+      <c r="A93" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="C93" s="32" t="n">
+        <v>20.667</v>
+      </c>
+      <c r="D93" s="32" t="n">
+        <v>19.95</v>
+      </c>
+      <c r="E93" s="32" t="n">
+        <v>20.067</v>
+      </c>
+      <c r="F93" s="32" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G93" s="32" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="H93" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I93" s="32" t="inlineStr"/>
+      <c r="J93" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P93" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q93" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B94" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C94" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D94" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E94" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F94" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G94" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H94" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I94" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J94" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K94" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L94" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M94" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N94" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O94" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P94" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q94" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C94" s="32" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D94" s="32" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="E94" s="32" t="n">
+        <v>10.733</v>
+      </c>
+      <c r="F94" s="32" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G94" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="H94" s="33" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="inlineStr"/>
+      <c r="J94" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P94" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q94" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>16.2</v>
       </c>
       <c r="C95" s="32" t="n">
-        <v>85.2</v>
+        <v>14.233</v>
       </c>
       <c r="D95" s="32" t="n">
-        <v>84.90000000000001</v>
+        <v>14.7</v>
       </c>
       <c r="E95" s="32" t="n">
-        <v>85.867</v>
+        <v>14.067</v>
       </c>
       <c r="F95" s="32" t="n">
-        <v>89.09999999999999</v>
+        <v>16.2</v>
       </c>
       <c r="G95" s="32" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="H95" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I95" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J95" s="33" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="K95" s="32" t="n">
-        <v>86.59999999999999</v>
-      </c>
-      <c r="L95" s="32" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="M95" s="32" t="n">
-        <v>88.69199999999999</v>
-      </c>
-      <c r="N95" s="32" t="n">
-        <v>86.889</v>
-      </c>
-      <c r="O95" s="32" t="n">
-        <v>89.25</v>
-      </c>
-      <c r="P95" s="32" t="n">
-        <v>87.5</v>
+        <v>15</v>
+      </c>
+      <c r="H95" s="33" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr"/>
+      <c r="J95" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P95" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q95" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="31" t="inlineStr">
-        <is>
-          <t>Off Rtg</t>
-        </is>
-      </c>
-      <c r="B96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="C96" s="32" t="n">
-        <v>107.942</v>
-      </c>
-      <c r="D96" s="32" t="n">
-        <v>105.587</v>
-      </c>
-      <c r="E96" s="32" t="n">
-        <v>105.509</v>
-      </c>
-      <c r="F96" s="32" t="n">
-        <v>109.659</v>
-      </c>
-      <c r="G96" s="32" t="n">
-        <v>115.565</v>
-      </c>
-      <c r="H96" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I96" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J96" s="33" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="K96" s="32" t="n">
-        <v>104.421</v>
-      </c>
-      <c r="L96" s="32" t="n">
-        <v>105.506</v>
-      </c>
-      <c r="M96" s="32" t="n">
-        <v>108.132</v>
-      </c>
-      <c r="N96" s="32" t="n">
-        <v>105.56</v>
-      </c>
-      <c r="O96" s="32" t="n">
-        <v>108.561</v>
-      </c>
-      <c r="P96" s="32" t="n">
-        <v>105.506</v>
-      </c>
-      <c r="Q96" s="34" t="inlineStr">
-        <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>eFG%</t>
-        </is>
-      </c>
-      <c r="B97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="C97" s="32" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="D97" s="32" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="E97" s="32" t="n">
-        <v>0.535</v>
-      </c>
-      <c r="F97" s="32" t="n">
-        <v>0.5570000000000001</v>
-      </c>
-      <c r="G97" s="32" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="H97" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I97" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J97" s="33" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K97" s="32" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="L97" s="32" t="n">
-        <v>0.529</v>
-      </c>
-      <c r="M97" s="32" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N97" s="32" t="n">
-        <v>0.523</v>
-      </c>
-      <c r="O97" s="32" t="n">
-        <v>0.535</v>
-      </c>
-      <c r="P97" s="32" t="n">
-        <v>0.529</v>
-      </c>
-      <c r="Q97" s="34" t="inlineStr">
-        <is>
-          <t>Opp eFG%</t>
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>Minnesota Lynx offense vs Los Angeles Sparks defense</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="31" t="inlineStr">
-        <is>
-          <t>2PT%</t>
-        </is>
-      </c>
-      <c r="B98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="C98" s="32" t="n">
-        <v>0.534</v>
-      </c>
-      <c r="D98" s="32" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="E98" s="32" t="n">
-        <v>0.549</v>
-      </c>
-      <c r="F98" s="32" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="G98" s="32" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="H98" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I98" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J98" s="33" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="K98" s="32" t="n">
-        <v>0.531</v>
-      </c>
-      <c r="L98" s="32" t="n">
-        <v>0.576</v>
-      </c>
-      <c r="M98" s="32" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="N98" s="32" t="n">
-        <v>0.513</v>
-      </c>
-      <c r="O98" s="32" t="n">
-        <v>0.524</v>
-      </c>
-      <c r="P98" s="32" t="n">
-        <v>0.576</v>
-      </c>
-      <c r="Q98" s="34" t="inlineStr">
-        <is>
-          <t>Opp 2PT%</t>
+      <c r="A98" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F98" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G98" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H98" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I98" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J98" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K98" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L98" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M98" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N98" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O98" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P98" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q98" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>0.374</v>
+        <v>85.2</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>0.343</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>0.347</v>
+        <v>85.867</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>0.373</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>0.382</v>
+        <v>94.2</v>
       </c>
       <c r="H99" s="36" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J99" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J99" s="33" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="K99" s="32" t="n">
-        <v>0.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="L99" s="32" t="n">
-        <v>0.296</v>
+        <v>87.5</v>
       </c>
       <c r="M99" s="32" t="n">
-        <v>0.33</v>
+        <v>88.69199999999999</v>
       </c>
       <c r="N99" s="32" t="n">
-        <v>0.352</v>
+        <v>86.889</v>
       </c>
       <c r="O99" s="32" t="n">
-        <v>0.365</v>
+        <v>89.25</v>
       </c>
       <c r="P99" s="32" t="n">
-        <v>0.296</v>
+        <v>87.5</v>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp PPG</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>Off Rtg</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.744</v>
+        <v>107.942</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.749</v>
+        <v>105.587</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.779</v>
+        <v>105.509</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.767</v>
+        <v>109.659</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.842</v>
+        <v>115.565</v>
       </c>
       <c r="H100" s="36" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I100" s="32" t="inlineStr"/>
-      <c r="J100" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P100" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J100" s="33" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="n">
+        <v>104.421</v>
+      </c>
+      <c r="L100" s="32" t="n">
+        <v>105.506</v>
+      </c>
+      <c r="M100" s="32" t="n">
+        <v>108.132</v>
+      </c>
+      <c r="N100" s="32" t="n">
+        <v>105.56</v>
+      </c>
+      <c r="O100" s="32" t="n">
+        <v>108.561</v>
+      </c>
+      <c r="P100" s="32" t="n">
+        <v>105.506</v>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>eFG%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>79.247</v>
+        <v>0.544</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>80.62</v>
+        <v>0.533</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>81.736</v>
+        <v>0.535</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>81.724</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>82.304</v>
-      </c>
-      <c r="H101" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr"/>
-      <c r="J101" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P101" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.579</v>
+      </c>
+      <c r="H101" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J101" s="33" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="L101" s="32" t="n">
+        <v>0.529</v>
+      </c>
+      <c r="M101" s="32" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N101" s="32" t="n">
+        <v>0.523</v>
+      </c>
+      <c r="O101" s="32" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="P101" s="32" t="n">
+        <v>0.529</v>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>2PT%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.591</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.57</v>
+        <v>0.534</v>
       </c>
       <c r="D102" s="32" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E102" s="32" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="F102" s="32" t="n">
         <v>0.5610000000000001</v>
       </c>
-      <c r="E102" s="32" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="F102" s="32" t="n">
-        <v>0.591</v>
-      </c>
       <c r="G102" s="32" t="n">
-        <v>0.613</v>
+        <v>0.582</v>
       </c>
       <c r="H102" s="36" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="I102" s="32" t="inlineStr"/>
-      <c r="J102" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P102" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I102" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J102" s="33" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="L102" s="32" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="M102" s="32" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="N102" s="32" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="O102" s="32" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="P102" s="32" t="n">
+        <v>0.576</v>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.255</v>
+        <v>0.374</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.253</v>
+        <v>0.343</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.245</v>
+        <v>0.347</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.265</v>
+        <v>0.373</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.287</v>
+        <v>0.382</v>
       </c>
       <c r="H103" s="36" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I103" s="32" t="inlineStr"/>
-      <c r="J103" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I103" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J103" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L103" s="32" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="M103" s="32" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="N103" s="32" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="O103" s="32" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <v>0.296</v>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>REB</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>34.9</v>
+        <v>0.744</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>36.05</v>
+        <v>0.749</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>36.467</v>
+        <v>0.779</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>37.6</v>
+        <v>0.767</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>40.4</v>
+        <v>0.842</v>
       </c>
       <c r="H104" s="36" t="inlineStr">
         <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I104" s="32" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J104" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K104" s="32" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="L104" s="32" t="n">
-        <v>34.375</v>
-      </c>
-      <c r="M104" s="32" t="n">
-        <v>37.538</v>
-      </c>
-      <c r="N104" s="32" t="n">
-        <v>36.389</v>
-      </c>
-      <c r="O104" s="32" t="n">
-        <v>35.357</v>
-      </c>
-      <c r="P104" s="32" t="n">
-        <v>34.375</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="inlineStr"/>
+      <c r="J104" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P104" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp REB</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>AST</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>21.533</v>
+        <v>79.247</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>21.1</v>
+        <v>80.62</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>20.867</v>
+        <v>81.736</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>21.1</v>
+        <v>81.724</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="H105" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
+        <v>82.304</v>
+      </c>
+      <c r="H105" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -2727,37 +2451,37 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp AST</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>BLK+STL</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>12.567</v>
+        <v>0.57</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>13.05</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>12.867</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>13</v>
+        <v>0.591</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>14.2</v>
+        <v>0.613</v>
       </c>
       <c r="H106" s="36" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I106" s="32" t="inlineStr"/>
@@ -2798,37 +2522,37 @@
       </c>
       <c r="Q106" s="34" t="inlineStr">
         <is>
-          <t>Opp BLK+STL</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="C107" s="32" t="n">
-        <v>12.733</v>
+        <v>0.255</v>
       </c>
       <c r="D107" s="32" t="n">
-        <v>13.35</v>
+        <v>0.253</v>
       </c>
       <c r="E107" s="32" t="n">
-        <v>13.733</v>
+        <v>0.245</v>
       </c>
       <c r="F107" s="32" t="n">
-        <v>14.8</v>
+        <v>0.265</v>
       </c>
       <c r="G107" s="32" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H107" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>0.287</v>
+      </c>
+      <c r="H107" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I107" s="32" t="inlineStr"/>
@@ -2868,6 +2592,282 @@
         </is>
       </c>
       <c r="Q107" s="34" t="inlineStr">
+        <is>
+          <t>Opp OREB%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="31" t="inlineStr">
+        <is>
+          <t>REB</t>
+        </is>
+      </c>
+      <c r="B108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="C108" s="32" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="D108" s="32" t="n">
+        <v>36.05</v>
+      </c>
+      <c r="E108" s="32" t="n">
+        <v>36.467</v>
+      </c>
+      <c r="F108" s="32" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G108" s="32" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="H108" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J108" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K108" s="32" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="L108" s="32" t="n">
+        <v>34.375</v>
+      </c>
+      <c r="M108" s="32" t="n">
+        <v>37.538</v>
+      </c>
+      <c r="N108" s="32" t="n">
+        <v>36.389</v>
+      </c>
+      <c r="O108" s="32" t="n">
+        <v>35.357</v>
+      </c>
+      <c r="P108" s="32" t="n">
+        <v>34.375</v>
+      </c>
+      <c r="Q108" s="34" t="inlineStr">
+        <is>
+          <t>Opp REB</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="31" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="B109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="C109" s="32" t="n">
+        <v>21.533</v>
+      </c>
+      <c r="D109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="E109" s="32" t="n">
+        <v>20.867</v>
+      </c>
+      <c r="F109" s="32" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G109" s="32" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H109" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I109" s="32" t="inlineStr"/>
+      <c r="J109" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P109" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q109" s="34" t="inlineStr">
+        <is>
+          <t>Opp AST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="31" t="inlineStr">
+        <is>
+          <t>BLK+STL</t>
+        </is>
+      </c>
+      <c r="B110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C110" s="32" t="n">
+        <v>12.567</v>
+      </c>
+      <c r="D110" s="32" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="E110" s="32" t="n">
+        <v>12.867</v>
+      </c>
+      <c r="F110" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G110" s="32" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H110" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="inlineStr"/>
+      <c r="J110" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P110" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q110" s="34" t="inlineStr">
+        <is>
+          <t>Opp BLK+STL</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="31" t="inlineStr">
+        <is>
+          <t>TOV</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C111" s="32" t="n">
+        <v>12.733</v>
+      </c>
+      <c r="D111" s="32" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="E111" s="32" t="n">
+        <v>13.733</v>
+      </c>
+      <c r="F111" s="32" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G111" s="32" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H111" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I111" s="32" t="inlineStr"/>
+      <c r="J111" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P111" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q111" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>
@@ -5048,13 +5048,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5792</v>
+        <v>0.5769</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-138</v>
+        <v>-136</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 57.9% (fair -138). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5090,37 +5090,37 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>New York Liberty @ Dallas Wings</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Dallas Wings -1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5193</v>
+        <v>0.5416</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-108</v>
+        <v>-118</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5171,22 +5171,22 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings -1.5</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5369</v>
+        <v>0.5696</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-116</v>
+        <v>-132</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-104</v>
+        <v>-117</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 57.0% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5227,32 +5227,32 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Washington Mystics -4.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5615</v>
+        <v>0.5349</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-128</v>
+        <v>-115</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5453,10 +5453,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4397</v>
+        <v>0.4355</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>127</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +127). Your call.</t>
+          <t>Model 43.5% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5519,13 +5519,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5603</v>
+        <v>0.5645</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-127</v>
+        <v>-130</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-127</v>
+        <v>-130</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 56.0% (fair -127). Your call.</t>
+          <t>Model 56.5% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5585,7 +5585,7 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4451</v>
+        <v>0.4448</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>125</v>
@@ -5651,7 +5651,7 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4731</v>
+        <v>0.4735</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>111</v>
@@ -5681,7 +5681,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5717,7 +5717,7 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3943</v>
+        <v>0.3935</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>154</v>
@@ -5783,7 +5783,7 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6057</v>
+        <v>0.6065</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>-154</v>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 60.6% (fair -154). Your call.</t>
+          <t>Model 60.7% (fair -154). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6062,7 +6062,7 @@
         <v>-146</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6118,17 +6118,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 171.5</t>
+          <t>Over 172.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6167891999123074</v>
+        <v>0.5941506978584125</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-161</v>
+        <v>-146</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -6152,7 +6152,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 59.4% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -6184,17 +6184,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 171.5</t>
+          <t>Under 172.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3832108000876926</v>
+        <v>0.4058493021415875</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>113</v>
+        <v>-101</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 40.6% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -6250,17 +6250,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -2.5</t>
+          <t>Chicago Sky -3</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5166439410560739</v>
+        <v>0.5009423824631134</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-107</v>
+        <v>-100</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -6316,14 +6316,14 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +2.5</t>
+          <t>Seattle Storm +3</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4833560589439261</v>
+        <v>0.4676576175368866</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>108</v>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6518,13 +6518,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4969</v>
+        <v>0.4988266420434531</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -6548,7 +6548,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -6584,10 +6584,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5031</v>
+        <v>0.5011733579565469</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-101</v>
+        <v>-100</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>100</v>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -6650,13 +6650,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4799</v>
+        <v>0.4852</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -6680,7 +6680,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -6716,13 +6716,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5201</v>
+        <v>0.5147999999999999</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-108</v>
+        <v>-103</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -6788,7 +6788,7 @@
         <v>124</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -6910,17 +6910,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Over 169</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5193</v>
+        <v>0.5503202853659634</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-108</v>
+        <v>-122</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -6944,7 +6944,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6976,14 +6976,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 169.5</t>
+          <t>Under 169</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4807</v>
+        <v>0.4263797146340366</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>104</v>
@@ -7010,7 +7010,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 42.6% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -7118,7 +7118,7 @@
         <v>-133</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -7310,13 +7310,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5792</v>
+        <v>0.5769</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-138</v>
+        <v>-136</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -7340,7 +7340,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 57.9% (fair -138). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -7376,10 +7376,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4208</v>
+        <v>0.4231</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>-110</v>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 42.1% (fair +138). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -7442,10 +7442,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5313</v>
+        <v>0.5349</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>-110</v>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 53.1% (fair -113). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -7508,13 +7508,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4687</v>
+        <v>0.4651</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-106</v>
+        <v>100</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 46.9% (fair +113). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -7574,13 +7574,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4385</v>
+        <v>0.4304</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -7604,7 +7604,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 43.9% (fair +128). Your call.</t>
+          <t>Model 43.0% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -7640,13 +7640,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5615</v>
+        <v>0.5696</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-128</v>
+        <v>-132</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-115</v>
+        <v>-117</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 57.0% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -7838,10 +7838,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5369</v>
+        <v>0.5416</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-116</v>
+        <v>-118</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>-104</v>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -7904,13 +7904,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4631</v>
+        <v>0.4584</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -8249,7 +8249,7 @@
         <v>243</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>

</xml_diff>

<commit_message>
data: hourly update 2026-07-15 14:56Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-15.xlsx
+++ b/data/output/workbook/2026-07-15.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 03:21</t>
+          <t>2026-07-15 10:55</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5044,14 +5044,14 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 165.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5769</v>
+        <v>0.5934</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-136</v>
+        <v>-146</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>-104</v>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5114,13 +5114,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5416</v>
+        <v>0.5392</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-118</v>
+        <v>-117</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5180,13 +5180,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5696</v>
+        <v>0.5704</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-132</v>
+        <v>-133</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -132). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5227,32 +5227,32 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics -4.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5359</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>-115</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5285,9 +5285,75 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>New York Liberty @ Dallas Wings</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Over 175.5</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0.5402</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-117</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I9" s="13">
+        <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF($H$9="","",$F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF($H$9="","",MAX(0,($F$9*IF($H$9&lt;0,-100/$H$9,$H$9/100)-(1-$F$9))/IF($H$9&lt;0,-100/$H$9,$H$9/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>IF($H$9="","",ROUND(MIN($K$9,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M9" s="12">
+        <f>IF($J$9="","",IF($J$9&lt;0,"Pass",IF($J$9&lt;'Settings'!$B$4,"Thin",IF($J$9&lt;0.06,"✅ Sharp band",IF($J$9&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.0% (fair -117). Your call.</t>
+        </is>
+      </c>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="16">
+        <f>IF(OR($H$9="",$O$9=""),"",(1+IF($H$9&lt;0,-100/$H$9,$H$9/100))/(1+IF($O$9&lt;0,-100/$O$9,$O$9/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J8">
+  <conditionalFormatting sqref="J5:J9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -5453,13 +5519,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4355</v>
+        <v>0.4297</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5483,7 +5549,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5519,13 +5585,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5645</v>
+        <v>0.5703</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-130</v>
+        <v>-133</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-130</v>
+        <v>-132</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5549,7 +5615,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5581,17 +5647,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 10</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4448</v>
+        <v>0.4641</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-110</v>
+        <v>108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5615,7 +5681,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 46.4% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5647,17 +5713,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 10</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4735</v>
+        <v>0.5359</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>111</v>
+        <v>-115</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5681,7 +5747,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5717,13 +5783,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3935</v>
+        <v>0.3831</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -5747,7 +5813,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 39.4% (fair +154). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5783,13 +5849,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6065</v>
+        <v>0.6169</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-154</v>
+        <v>-161</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-170</v>
+        <v>-160</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -5813,7 +5879,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -154). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -5996,7 +6062,7 @@
         <v>146</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -6062,7 +6128,7 @@
         <v>-146</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6194,7 +6260,7 @@
         <v>146</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-101</v>
+        <v>102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -6250,17 +6316,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -3</t>
+          <t>Chicago Sky -5.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5009423824631134</v>
+        <v>0.4228968214967185</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-100</v>
+        <v>136</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -6284,7 +6350,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -6316,17 +6382,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +3</t>
+          <t>Seattle Storm +5.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4676576175368866</v>
+        <v>0.5771031785032815</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>114</v>
+        <v>-136</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -6350,7 +6416,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6392,7 +6458,7 @@
         <v>1157</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -6458,7 +6524,7 @@
         <v>-1157</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -6514,17 +6580,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Over 182.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4988266420434531</v>
+        <v>0.5222822354138622</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>100</v>
+        <v>-109</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -6548,7 +6614,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -6580,17 +6646,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 183.5</t>
+          <t>Under 182.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5011733579565469</v>
+        <v>0.4777177645861378</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-100</v>
+        <v>109</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -6614,7 +6680,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -6650,13 +6716,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4852</v>
+        <v>0.4789631974236769</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -6680,7 +6746,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -6716,13 +6782,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5147999999999999</v>
+        <v>0.5210368025763231</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-106</v>
+        <v>-109</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-103</v>
+        <v>-104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -6746,7 +6812,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -6782,13 +6848,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.445452</v>
+        <v>0.4553</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -6812,7 +6878,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +124). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -6848,10 +6914,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.554548</v>
+        <v>0.5447</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-124</v>
+        <v>-120</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>-115</v>
@@ -6878,7 +6944,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -124). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -6910,17 +6976,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 169</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5503202853659634</v>
+        <v>0.5850016819596556</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-122</v>
+        <v>-141</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -6944,7 +7010,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -6976,17 +7042,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 169</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4263797146340366</v>
+        <v>0.4149983180403444</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>104</v>
+        <v>-105</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -7010,7 +7076,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -7042,17 +7108,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -3.5</t>
+          <t>Indiana Fever -3</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4284526556424175</v>
+        <v>0.4439567427023119</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -7076,7 +7142,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.8% (fair +133). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -7108,17 +7174,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +3.5</t>
+          <t>Golden State Valkyries +3</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5715473443575825</v>
+        <v>0.5249432572976881</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-133</v>
+        <v>-111</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -7142,7 +7208,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.2% (fair -133). Your call.</t>
+          <t>Model 52.5% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -7250,7 +7316,7 @@
         <v>-220</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-120</v>
+        <v>-110</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -7306,14 +7372,14 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 165.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5769</v>
+        <v>0.5934</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-136</v>
+        <v>-146</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>-104</v>
@@ -7340,7 +7406,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -7372,17 +7438,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 166.5</t>
+          <t>Under 165.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4231</v>
+        <v>0.4066</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -7406,7 +7472,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -7438,17 +7504,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics -4.5</t>
+          <t>Washington Mystics -5.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5349</v>
+        <v>0.5269943569232249</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-115</v>
+        <v>-111</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -7472,7 +7538,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -7504,17 +7570,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +4.5</t>
+          <t>Portland Fire +5.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4651</v>
+        <v>0.4730056430767751</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -7538,7 +7604,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -7574,13 +7640,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4304</v>
+        <v>0.4296</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -7604,7 +7670,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 43.0% (fair +132). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -7640,13 +7706,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5696</v>
+        <v>0.5704</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-132</v>
+        <v>-133</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -7670,7 +7736,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -132). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -7706,10 +7772,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5341</v>
+        <v>0.5402</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-115</v>
+        <v>-117</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>-110</v>
@@ -7736,7 +7802,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -7772,13 +7838,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4659</v>
+        <v>0.4598</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>-106</v>
+        <v>104</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -7802,7 +7868,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -7838,13 +7904,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5416</v>
+        <v>0.5392</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-118</v>
+        <v>-117</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -7868,7 +7934,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -7904,10 +7970,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4584</v>
+        <v>0.4608</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>100</v>
@@ -7934,7 +8000,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -8117,7 +8183,7 @@
         <v>243</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8447,7 +8513,7 @@
         <v>130</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-208</v>
+        <v>-222</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>

</xml_diff>

<commit_message>
data: hourly update 2026-07-15 16:28Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-15.xlsx
+++ b/data/output/workbook/2026-07-15.xlsx
@@ -395,7 +395,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="12687300"/>
+    <ext cx="10125075" cy="12125325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 10:55</t>
+          <t>2026-07-15 12:28</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q110"/>
+  <dimension ref="A1:Q106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2903,501 +2903,773 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries offense vs Indiana Fever defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F77" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H77" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L77" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M77" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N77" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O77" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P77" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q77" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="n">
+        <v>86.77800000000001</v>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>80.55</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>90</v>
+      </c>
+      <c r="H78" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J78" s="33" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>91</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>88.143</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>83.57899999999999</v>
+      </c>
+      <c r="O78" s="32" t="n">
+        <v>83.517</v>
+      </c>
+      <c r="P78" s="32" t="n">
+        <v>89</v>
+      </c>
+      <c r="Q78" s="34" t="inlineStr">
+        <is>
+          <t>Opp PPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="n">
+        <v>107.652</v>
+      </c>
+      <c r="C79" s="32" t="n">
+        <v>103.937</v>
+      </c>
+      <c r="D79" s="32" t="n">
+        <v>102.955</v>
+      </c>
+      <c r="E79" s="32" t="n">
+        <v>101.595</v>
+      </c>
+      <c r="F79" s="32" t="n">
+        <v>106.892</v>
+      </c>
+      <c r="G79" s="32" t="n">
+        <v>111.51</v>
+      </c>
+      <c r="H79" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J79" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="n">
+        <v>101.505</v>
+      </c>
+      <c r="L79" s="32" t="n">
+        <v>105.886</v>
+      </c>
+      <c r="M79" s="32" t="n">
+        <v>104.078</v>
+      </c>
+      <c r="N79" s="32" t="n">
+        <v>100.581</v>
+      </c>
+      <c r="O79" s="32" t="n">
+        <v>102.673</v>
+      </c>
+      <c r="P79" s="32" t="n">
+        <v>104.372</v>
+      </c>
+      <c r="Q79" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
+        </is>
+      </c>
+    </row>
     <row r="80">
-      <c r="A80" s="29" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries offense vs Indiana Fever defense</t>
+      <c r="A80" s="31" t="inlineStr">
+        <is>
+          <t>eFG%</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="C80" s="32" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="D80" s="32" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="E80" s="32" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="F80" s="32" t="n">
+        <v>0.499</v>
+      </c>
+      <c r="G80" s="32" t="n">
+        <v>0.519</v>
+      </c>
+      <c r="H80" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="L80" s="32" t="n">
+        <v>0.523</v>
+      </c>
+      <c r="M80" s="32" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="N80" s="32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="O80" s="32" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="Q80" s="34" t="inlineStr">
+        <is>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B81" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C81" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D81" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E81" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F81" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G81" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H81" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I81" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J81" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K81" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L81" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M81" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N81" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O81" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P81" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q81" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>2PT%</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="E81" s="32" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="F81" s="32" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="G81" s="32" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="H81" s="33" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="L81" s="32" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="M81" s="32" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="N81" s="32" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="Q81" s="34" t="inlineStr">
+        <is>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B82" s="32" t="n">
-        <v>86.77800000000001</v>
+        <v>0.382</v>
       </c>
       <c r="C82" s="32" t="n">
-        <v>79.3</v>
+        <v>0.36</v>
       </c>
       <c r="D82" s="32" t="n">
-        <v>80.55</v>
+        <v>0.363</v>
       </c>
       <c r="E82" s="32" t="n">
-        <v>80.59999999999999</v>
+        <v>0.353</v>
       </c>
       <c r="F82" s="32" t="n">
-        <v>85.5</v>
+        <v>0.394</v>
       </c>
       <c r="G82" s="32" t="n">
-        <v>90</v>
+        <v>0.411</v>
       </c>
       <c r="H82" s="36" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="I82" s="32" t="inlineStr">
         <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J82" s="33" t="inlineStr">
-        <is>
-          <t>10th</t>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J82" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
         </is>
       </c>
       <c r="K82" s="32" t="n">
-        <v>84.59999999999999</v>
+        <v>0.308</v>
       </c>
       <c r="L82" s="32" t="n">
-        <v>91</v>
+        <v>0.332</v>
       </c>
       <c r="M82" s="32" t="n">
-        <v>88.143</v>
+        <v>0.34</v>
       </c>
       <c r="N82" s="32" t="n">
-        <v>83.57899999999999</v>
+        <v>0.311</v>
       </c>
       <c r="O82" s="32" t="n">
-        <v>83.517</v>
+        <v>0.346</v>
       </c>
       <c r="P82" s="32" t="n">
-        <v>89</v>
+        <v>0.321</v>
       </c>
       <c r="Q82" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B83" s="32" t="n">
-        <v>107.652</v>
+        <v>0.762</v>
       </c>
       <c r="C83" s="32" t="n">
-        <v>103.937</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D83" s="32" t="n">
-        <v>102.955</v>
+        <v>0.79</v>
       </c>
       <c r="E83" s="32" t="n">
-        <v>101.595</v>
+        <v>0.777</v>
       </c>
       <c r="F83" s="32" t="n">
-        <v>106.892</v>
+        <v>0.764</v>
       </c>
       <c r="G83" s="32" t="n">
-        <v>111.51</v>
-      </c>
-      <c r="H83" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I83" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J83" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="K83" s="32" t="n">
-        <v>101.505</v>
-      </c>
-      <c r="L83" s="32" t="n">
-        <v>105.886</v>
-      </c>
-      <c r="M83" s="32" t="n">
-        <v>104.078</v>
-      </c>
-      <c r="N83" s="32" t="n">
-        <v>100.581</v>
-      </c>
-      <c r="O83" s="32" t="n">
-        <v>102.673</v>
-      </c>
-      <c r="P83" s="32" t="n">
-        <v>104.372</v>
+        <v>0.747</v>
+      </c>
+      <c r="H83" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I83" s="32" t="inlineStr"/>
+      <c r="J83" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P83" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q83" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B84" s="32" t="n">
-        <v>0.496</v>
+        <v>80.818</v>
       </c>
       <c r="C84" s="32" t="n">
-        <v>0.494</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D84" s="32" t="n">
-        <v>0.493</v>
+        <v>78.298</v>
       </c>
       <c r="E84" s="32" t="n">
-        <v>0.476</v>
+        <v>79.42400000000001</v>
       </c>
       <c r="F84" s="32" t="n">
-        <v>0.499</v>
+        <v>80.13200000000001</v>
       </c>
       <c r="G84" s="32" t="n">
-        <v>0.519</v>
+        <v>80.968</v>
       </c>
       <c r="H84" s="35" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>6th</t>
         </is>
       </c>
       <c r="I84" s="32" t="inlineStr"/>
-      <c r="J84" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K84" s="32" t="n">
-        <v>0.474</v>
-      </c>
-      <c r="L84" s="32" t="n">
-        <v>0.523</v>
-      </c>
-      <c r="M84" s="32" t="n">
-        <v>0.526</v>
-      </c>
-      <c r="N84" s="32" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="O84" s="32" t="n">
-        <v>0.526</v>
-      </c>
-      <c r="P84" s="32" t="n">
-        <v>0.52</v>
+      <c r="J84" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P84" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q84" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B85" s="32" t="n">
-        <v>0.43</v>
+        <v>0.539</v>
       </c>
       <c r="C85" s="32" t="n">
-        <v>0.456</v>
+        <v>0.541</v>
       </c>
       <c r="D85" s="32" t="n">
-        <v>0.456</v>
+        <v>0.538</v>
       </c>
       <c r="E85" s="32" t="n">
-        <v>0.435</v>
+        <v>0.521</v>
       </c>
       <c r="F85" s="32" t="n">
-        <v>0.427</v>
+        <v>0.54</v>
       </c>
       <c r="G85" s="32" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="H85" s="33" t="inlineStr">
-        <is>
-          <t>14th</t>
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="H85" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
         </is>
       </c>
       <c r="I85" s="32" t="inlineStr"/>
-      <c r="J85" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="K85" s="32" t="n">
-        <v>0.475</v>
-      </c>
-      <c r="L85" s="32" t="n">
-        <v>0.527</v>
-      </c>
-      <c r="M85" s="32" t="n">
-        <v>0.531</v>
-      </c>
-      <c r="N85" s="32" t="n">
-        <v>0.524</v>
-      </c>
-      <c r="O85" s="32" t="n">
-        <v>0.525</v>
-      </c>
-      <c r="P85" s="32" t="n">
-        <v>0.53</v>
+      <c r="J85" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P85" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q85" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B86" s="32" t="n">
-        <v>0.382</v>
+        <v>0.27</v>
       </c>
       <c r="C86" s="32" t="n">
-        <v>0.36</v>
+        <v>0.244</v>
       </c>
       <c r="D86" s="32" t="n">
-        <v>0.363</v>
+        <v>0.25</v>
       </c>
       <c r="E86" s="32" t="n">
-        <v>0.353</v>
+        <v>0.264</v>
       </c>
       <c r="F86" s="32" t="n">
-        <v>0.394</v>
+        <v>0.264</v>
       </c>
       <c r="G86" s="32" t="n">
-        <v>0.411</v>
-      </c>
-      <c r="H86" s="36" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I86" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J86" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="K86" s="32" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="L86" s="32" t="n">
-        <v>0.332</v>
-      </c>
-      <c r="M86" s="32" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="N86" s="32" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="O86" s="32" t="n">
-        <v>0.346</v>
-      </c>
-      <c r="P86" s="32" t="n">
-        <v>0.321</v>
+        <v>0.258</v>
+      </c>
+      <c r="H86" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I86" s="32" t="inlineStr"/>
+      <c r="J86" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P86" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q86" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B87" s="32" t="n">
-        <v>0.762</v>
+        <v>33.778</v>
       </c>
       <c r="C87" s="32" t="n">
-        <v>0.8100000000000001</v>
+        <v>33.5</v>
       </c>
       <c r="D87" s="32" t="n">
-        <v>0.79</v>
+        <v>33.95</v>
       </c>
       <c r="E87" s="32" t="n">
-        <v>0.777</v>
+        <v>33.8</v>
       </c>
       <c r="F87" s="32" t="n">
-        <v>0.764</v>
+        <v>33.2</v>
       </c>
       <c r="G87" s="32" t="n">
-        <v>0.747</v>
-      </c>
-      <c r="H87" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>33.8</v>
+      </c>
+      <c r="H87" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I87" s="32" t="inlineStr"/>
-      <c r="J87" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P87" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J87" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="K87" s="32" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="L87" s="32" t="n">
+        <v>28.667</v>
+      </c>
+      <c r="M87" s="32" t="n">
+        <v>29.143</v>
+      </c>
+      <c r="N87" s="32" t="n">
+        <v>29.842</v>
+      </c>
+      <c r="O87" s="32" t="n">
+        <v>30.31</v>
+      </c>
+      <c r="P87" s="32" t="n">
+        <v>29.625</v>
       </c>
       <c r="Q87" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B88" s="32" t="n">
-        <v>80.818</v>
+        <v>19.444</v>
       </c>
       <c r="C88" s="32" t="n">
-        <v>76.40000000000001</v>
+        <v>19.033</v>
       </c>
       <c r="D88" s="32" t="n">
-        <v>78.298</v>
+        <v>19.4</v>
       </c>
       <c r="E88" s="32" t="n">
-        <v>79.42400000000001</v>
+        <v>19</v>
       </c>
       <c r="F88" s="32" t="n">
-        <v>80.13200000000001</v>
+        <v>19.7</v>
       </c>
       <c r="G88" s="32" t="n">
-        <v>80.968</v>
+        <v>21.4</v>
       </c>
       <c r="H88" s="35" t="inlineStr">
         <is>
@@ -3442,37 +3714,37 @@
       </c>
       <c r="Q88" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B89" s="32" t="n">
-        <v>0.539</v>
+        <v>11.444</v>
       </c>
       <c r="C89" s="32" t="n">
-        <v>0.541</v>
+        <v>10.233</v>
       </c>
       <c r="D89" s="32" t="n">
-        <v>0.538</v>
+        <v>11.1</v>
       </c>
       <c r="E89" s="32" t="n">
-        <v>0.521</v>
+        <v>11.533</v>
       </c>
       <c r="F89" s="32" t="n">
-        <v>0.54</v>
+        <v>11.5</v>
       </c>
       <c r="G89" s="32" t="n">
-        <v>0.5580000000000001</v>
+        <v>11</v>
       </c>
       <c r="H89" s="35" t="inlineStr">
         <is>
-          <t>7th</t>
+          <t>9th</t>
         </is>
       </c>
       <c r="I89" s="32" t="inlineStr"/>
@@ -3513,37 +3785,37 @@
       </c>
       <c r="Q89" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B90" s="32" t="n">
-        <v>0.27</v>
+        <v>10</v>
       </c>
       <c r="C90" s="32" t="n">
-        <v>0.244</v>
+        <v>11.1</v>
       </c>
       <c r="D90" s="32" t="n">
-        <v>0.25</v>
+        <v>11.75</v>
       </c>
       <c r="E90" s="32" t="n">
-        <v>0.264</v>
+        <v>11.6</v>
       </c>
       <c r="F90" s="32" t="n">
-        <v>0.264</v>
+        <v>10.2</v>
       </c>
       <c r="G90" s="32" t="n">
-        <v>0.258</v>
-      </c>
-      <c r="H90" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>9.4</v>
+      </c>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="I90" s="32" t="inlineStr"/>
@@ -3584,773 +3856,777 @@
       </c>
       <c r="Q90" s="34" t="inlineStr">
         <is>
-          <t>Opp OREB%</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="31" t="inlineStr">
-        <is>
-          <t>REB</t>
-        </is>
-      </c>
-      <c r="B91" s="32" t="n">
-        <v>33.778</v>
-      </c>
-      <c r="C91" s="32" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="D91" s="32" t="n">
-        <v>33.95</v>
-      </c>
-      <c r="E91" s="32" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="F91" s="32" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="G91" s="32" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="H91" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I91" s="32" t="inlineStr"/>
-      <c r="J91" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="K91" s="32" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="L91" s="32" t="n">
-        <v>28.667</v>
-      </c>
-      <c r="M91" s="32" t="n">
-        <v>29.143</v>
-      </c>
-      <c r="N91" s="32" t="n">
-        <v>29.842</v>
-      </c>
-      <c r="O91" s="32" t="n">
-        <v>30.31</v>
-      </c>
-      <c r="P91" s="32" t="n">
-        <v>29.625</v>
-      </c>
-      <c r="Q91" s="34" t="inlineStr">
-        <is>
-          <t>Opp REB</t>
+          <t>Opp TOV</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="31" t="inlineStr">
-        <is>
-          <t>AST</t>
-        </is>
-      </c>
-      <c r="B92" s="32" t="n">
-        <v>19.444</v>
-      </c>
-      <c r="C92" s="32" t="n">
-        <v>19.033</v>
-      </c>
-      <c r="D92" s="32" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="E92" s="32" t="n">
-        <v>19</v>
-      </c>
-      <c r="F92" s="32" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="G92" s="32" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="H92" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I92" s="32" t="inlineStr"/>
-      <c r="J92" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P92" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q92" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>Indiana Fever offense vs Golden State Valkyries defense</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B93" s="32" t="n">
-        <v>11.444</v>
-      </c>
-      <c r="C93" s="32" t="n">
-        <v>10.233</v>
-      </c>
-      <c r="D93" s="32" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="E93" s="32" t="n">
-        <v>11.533</v>
-      </c>
-      <c r="F93" s="32" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G93" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="H93" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="I93" s="32" t="inlineStr"/>
-      <c r="J93" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P93" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q93" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
+      <c r="A93" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B93" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C93" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D93" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E93" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F93" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G93" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H93" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I93" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J93" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K93" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L93" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M93" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N93" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O93" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P93" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q93" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="31" t="inlineStr">
         <is>
-          <t>TOV</t>
+          <t>PPG</t>
         </is>
       </c>
       <c r="B94" s="32" t="n">
-        <v>10</v>
+        <v>93.22199999999999</v>
       </c>
       <c r="C94" s="32" t="n">
-        <v>11.1</v>
+        <v>86.8</v>
       </c>
       <c r="D94" s="32" t="n">
-        <v>11.75</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="E94" s="32" t="n">
-        <v>11.6</v>
+        <v>89.533</v>
       </c>
       <c r="F94" s="32" t="n">
-        <v>10.2</v>
+        <v>93.7</v>
       </c>
       <c r="G94" s="32" t="n">
-        <v>9.4</v>
+        <v>88.2</v>
       </c>
       <c r="H94" s="36" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="I94" s="32" t="inlineStr"/>
-      <c r="J94" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P94" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J94" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K94" s="32" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="L94" s="32" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="M94" s="32" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="N94" s="32" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="O94" s="32" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="P94" s="32" t="n">
+        <v>79.333</v>
       </c>
       <c r="Q94" s="34" t="inlineStr">
         <is>
-          <t>Opp TOV</t>
+          <t>Opp PPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>Off Rtg</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="C95" s="32" t="n">
+        <v>105.41</v>
+      </c>
+      <c r="D95" s="32" t="n">
+        <v>105.193</v>
+      </c>
+      <c r="E95" s="32" t="n">
+        <v>104.632</v>
+      </c>
+      <c r="F95" s="32" t="n">
+        <v>107.032</v>
+      </c>
+      <c r="G95" s="32" t="n">
+        <v>104.061</v>
+      </c>
+      <c r="H95" s="35" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="inlineStr"/>
+      <c r="J95" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="K95" s="32" t="n">
+        <v>99.15600000000001</v>
+      </c>
+      <c r="L95" s="32" t="n">
+        <v>99.73399999999999</v>
+      </c>
+      <c r="M95" s="32" t="n">
+        <v>101.464</v>
+      </c>
+      <c r="N95" s="32" t="n">
+        <v>99.227</v>
+      </c>
+      <c r="O95" s="32" t="n">
+        <v>99.539</v>
+      </c>
+      <c r="P95" s="32" t="n">
+        <v>99.908</v>
+      </c>
+      <c r="Q95" s="34" t="inlineStr">
+        <is>
+          <t>Opp Off Rtg</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="29" t="inlineStr">
-        <is>
-          <t>Indiana Fever offense vs Golden State Valkyries defense</t>
+      <c r="A96" s="31" t="inlineStr">
+        <is>
+          <t>eFG%</t>
+        </is>
+      </c>
+      <c r="B96" s="32" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="C96" s="32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D96" s="32" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="E96" s="32" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="F96" s="32" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="G96" s="32" t="n">
+        <v>0.499</v>
+      </c>
+      <c r="H96" s="35" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I96" s="32" t="inlineStr"/>
+      <c r="J96" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
+        </is>
+      </c>
+      <c r="K96" s="32" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L96" s="32" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="M96" s="32" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="N96" s="32" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="O96" s="32" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="P96" s="32" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="Q96" s="34" t="inlineStr">
+        <is>
+          <t>Opp eFG%</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B97" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C97" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D97" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E97" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F97" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G97" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H97" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I97" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J97" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K97" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L97" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M97" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N97" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O97" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P97" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q97" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A97" s="31" t="inlineStr">
+        <is>
+          <t>2PT%</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="C97" s="32" t="n">
+        <v>0.506</v>
+      </c>
+      <c r="D97" s="32" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="E97" s="32" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="F97" s="32" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="G97" s="32" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="H97" s="36" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="I97" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J97" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
+        </is>
+      </c>
+      <c r="K97" s="32" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L97" s="32" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="M97" s="32" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="N97" s="32" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="O97" s="32" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="P97" s="32" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="Q97" s="34" t="inlineStr">
+        <is>
+          <t>Opp 2PT%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="31" t="inlineStr">
         <is>
-          <t>PPG</t>
+          <t>3PT%</t>
         </is>
       </c>
       <c r="B98" s="32" t="n">
-        <v>93.22199999999999</v>
+        <v>0.327</v>
       </c>
       <c r="C98" s="32" t="n">
-        <v>86.8</v>
+        <v>0.346</v>
       </c>
       <c r="D98" s="32" t="n">
-        <v>88.09999999999999</v>
+        <v>0.331</v>
       </c>
       <c r="E98" s="32" t="n">
-        <v>89.533</v>
+        <v>0.324</v>
       </c>
       <c r="F98" s="32" t="n">
-        <v>93.7</v>
+        <v>0.335</v>
       </c>
       <c r="G98" s="32" t="n">
-        <v>88.2</v>
-      </c>
-      <c r="H98" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
+        <v>0.299</v>
+      </c>
+      <c r="H98" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I98" s="32" t="inlineStr"/>
       <c r="J98" s="35" t="inlineStr">
         <is>
-          <t>5th</t>
+          <t>9th</t>
         </is>
       </c>
       <c r="K98" s="32" t="n">
-        <v>79.2</v>
+        <v>0.329</v>
       </c>
       <c r="L98" s="32" t="n">
-        <v>78.90000000000001</v>
+        <v>0.346</v>
       </c>
       <c r="M98" s="32" t="n">
-        <v>79.59999999999999</v>
+        <v>0.347</v>
       </c>
       <c r="N98" s="32" t="n">
-        <v>76.95</v>
+        <v>0.333</v>
       </c>
       <c r="O98" s="32" t="n">
-        <v>76.2</v>
+        <v>0.316</v>
       </c>
       <c r="P98" s="32" t="n">
-        <v>79.333</v>
+        <v>0.353</v>
       </c>
       <c r="Q98" s="34" t="inlineStr">
         <is>
-          <t>Opp PPG</t>
+          <t>Opp 3PT%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
         <is>
-          <t>Off Rtg</t>
+          <t>FT%</t>
         </is>
       </c>
       <c r="B99" s="32" t="n">
-        <v>106.9</v>
+        <v>0.85</v>
       </c>
       <c r="C99" s="32" t="n">
-        <v>105.41</v>
+        <v>0.795</v>
       </c>
       <c r="D99" s="32" t="n">
-        <v>105.193</v>
+        <v>0.819</v>
       </c>
       <c r="E99" s="32" t="n">
-        <v>104.632</v>
+        <v>0.82</v>
       </c>
       <c r="F99" s="32" t="n">
-        <v>107.032</v>
+        <v>0.853</v>
       </c>
       <c r="G99" s="32" t="n">
-        <v>104.061</v>
-      </c>
-      <c r="H99" s="35" t="inlineStr">
-        <is>
-          <t>7th</t>
+        <v>0.882</v>
+      </c>
+      <c r="H99" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I99" s="32" t="inlineStr"/>
-      <c r="J99" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K99" s="32" t="n">
-        <v>99.15600000000001</v>
-      </c>
-      <c r="L99" s="32" t="n">
-        <v>99.73399999999999</v>
-      </c>
-      <c r="M99" s="32" t="n">
-        <v>101.464</v>
-      </c>
-      <c r="N99" s="32" t="n">
-        <v>99.227</v>
-      </c>
-      <c r="O99" s="32" t="n">
-        <v>99.539</v>
-      </c>
-      <c r="P99" s="32" t="n">
-        <v>99.908</v>
+      <c r="J99" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P99" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q99" s="34" t="inlineStr">
         <is>
-          <t>Opp Off Rtg</t>
+          <t>Opp FT%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
         <is>
-          <t>eFG%</t>
+          <t>Pace</t>
         </is>
       </c>
       <c r="B100" s="32" t="n">
-        <v>0.527</v>
+        <v>87.227</v>
       </c>
       <c r="C100" s="32" t="n">
-        <v>0.51</v>
+        <v>82.343</v>
       </c>
       <c r="D100" s="32" t="n">
-        <v>0.508</v>
+        <v>83.684</v>
       </c>
       <c r="E100" s="32" t="n">
-        <v>0.508</v>
+        <v>85.429</v>
       </c>
       <c r="F100" s="32" t="n">
-        <v>0.527</v>
+        <v>87.56</v>
       </c>
       <c r="G100" s="32" t="n">
-        <v>0.499</v>
-      </c>
-      <c r="H100" s="35" t="inlineStr">
-        <is>
-          <t>8th</t>
+        <v>84.768</v>
+      </c>
+      <c r="H100" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="I100" s="32" t="inlineStr"/>
-      <c r="J100" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="K100" s="32" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="L100" s="32" t="n">
-        <v>0.498</v>
-      </c>
-      <c r="M100" s="32" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="N100" s="32" t="n">
-        <v>0.482</v>
-      </c>
-      <c r="O100" s="32" t="n">
-        <v>0.479</v>
-      </c>
-      <c r="P100" s="32" t="n">
-        <v>0.496</v>
+      <c r="J100" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P100" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q100" s="34" t="inlineStr">
         <is>
-          <t>Opp eFG%</t>
+          <t>Opp Pace</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
         <is>
-          <t>2PT%</t>
+          <t>TS%</t>
         </is>
       </c>
       <c r="B101" s="32" t="n">
-        <v>0.546</v>
+        <v>0.588</v>
       </c>
       <c r="C101" s="32" t="n">
-        <v>0.506</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="D101" s="32" t="n">
-        <v>0.513</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="E101" s="32" t="n">
-        <v>0.517</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="F101" s="32" t="n">
-        <v>0.541</v>
+        <v>0.588</v>
       </c>
       <c r="G101" s="32" t="n">
-        <v>0.526</v>
+        <v>0.577</v>
       </c>
       <c r="H101" s="36" t="inlineStr">
         <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="I101" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J101" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="K101" s="32" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="L101" s="32" t="n">
-        <v>0.487</v>
-      </c>
-      <c r="M101" s="32" t="n">
-        <v>0.484</v>
-      </c>
-      <c r="N101" s="32" t="n">
-        <v>0.471</v>
-      </c>
-      <c r="O101" s="32" t="n">
-        <v>0.485</v>
-      </c>
-      <c r="P101" s="32" t="n">
-        <v>0.475</v>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="inlineStr"/>
+      <c r="J101" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P101" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q101" s="34" t="inlineStr">
         <is>
-          <t>Opp 2PT%</t>
+          <t>Opp TS%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
         <is>
-          <t>3PT%</t>
+          <t>OREB%</t>
         </is>
       </c>
       <c r="B102" s="32" t="n">
-        <v>0.327</v>
+        <v>0.251</v>
       </c>
       <c r="C102" s="32" t="n">
-        <v>0.346</v>
+        <v>0.278</v>
       </c>
       <c r="D102" s="32" t="n">
-        <v>0.331</v>
+        <v>0.272</v>
       </c>
       <c r="E102" s="32" t="n">
-        <v>0.324</v>
+        <v>0.281</v>
       </c>
       <c r="F102" s="32" t="n">
-        <v>0.335</v>
+        <v>0.273</v>
       </c>
       <c r="G102" s="32" t="n">
-        <v>0.299</v>
-      </c>
-      <c r="H102" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
+        <v>0.253</v>
+      </c>
+      <c r="H102" s="35" t="inlineStr">
+        <is>
+          <t>8th</t>
         </is>
       </c>
       <c r="I102" s="32" t="inlineStr"/>
-      <c r="J102" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="K102" s="32" t="n">
-        <v>0.329</v>
-      </c>
-      <c r="L102" s="32" t="n">
-        <v>0.346</v>
-      </c>
-      <c r="M102" s="32" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="N102" s="32" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O102" s="32" t="n">
-        <v>0.316</v>
-      </c>
-      <c r="P102" s="32" t="n">
-        <v>0.353</v>
+      <c r="J102" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P102" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q102" s="34" t="inlineStr">
         <is>
-          <t>Opp 3PT%</t>
+          <t>Opp OREB%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
         <is>
-          <t>FT%</t>
+          <t>REB</t>
         </is>
       </c>
       <c r="B103" s="32" t="n">
-        <v>0.85</v>
+        <v>33</v>
       </c>
       <c r="C103" s="32" t="n">
-        <v>0.795</v>
+        <v>33.433</v>
       </c>
       <c r="D103" s="32" t="n">
-        <v>0.819</v>
+        <v>33.2</v>
       </c>
       <c r="E103" s="32" t="n">
-        <v>0.82</v>
+        <v>33.933</v>
       </c>
       <c r="F103" s="32" t="n">
-        <v>0.853</v>
+        <v>33.7</v>
       </c>
       <c r="G103" s="32" t="n">
-        <v>0.882</v>
-      </c>
-      <c r="H103" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I103" s="32" t="inlineStr"/>
-      <c r="J103" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P103" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>33.6</v>
+      </c>
+      <c r="H103" s="35" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="I103" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J103" s="35" t="inlineStr">
+        <is>
+          <t>9th</t>
+        </is>
+      </c>
+      <c r="K103" s="32" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="L103" s="32" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="M103" s="32" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="N103" s="32" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="O103" s="32" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="P103" s="32" t="n">
+        <v>34.889</v>
       </c>
       <c r="Q103" s="34" t="inlineStr">
         <is>
-          <t>Opp FT%</t>
+          <t>Opp REB</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
         <is>
-          <t>Pace</t>
+          <t>AST</t>
         </is>
       </c>
       <c r="B104" s="32" t="n">
-        <v>87.227</v>
+        <v>22.556</v>
       </c>
       <c r="C104" s="32" t="n">
-        <v>82.343</v>
+        <v>20.567</v>
       </c>
       <c r="D104" s="32" t="n">
-        <v>83.684</v>
+        <v>20.45</v>
       </c>
       <c r="E104" s="32" t="n">
-        <v>85.429</v>
+        <v>20.733</v>
       </c>
       <c r="F104" s="32" t="n">
-        <v>87.56</v>
+        <v>22.4</v>
       </c>
       <c r="G104" s="32" t="n">
-        <v>84.768</v>
-      </c>
-      <c r="H104" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
+        <v>21.6</v>
+      </c>
+      <c r="H104" s="35" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I104" s="32" t="inlineStr"/>
@@ -4391,37 +4667,37 @@
       </c>
       <c r="Q104" s="34" t="inlineStr">
         <is>
-          <t>Opp Pace</t>
+          <t>Opp AST</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
         <is>
-          <t>TS%</t>
+          <t>BLK+STL</t>
         </is>
       </c>
       <c r="B105" s="32" t="n">
-        <v>0.588</v>
+        <v>11.333</v>
       </c>
       <c r="C105" s="32" t="n">
-        <v>0.5570000000000001</v>
+        <v>10</v>
       </c>
       <c r="D105" s="32" t="n">
-        <v>0.5620000000000001</v>
+        <v>10.05</v>
       </c>
       <c r="E105" s="32" t="n">
-        <v>0.5639999999999999</v>
+        <v>10.467</v>
       </c>
       <c r="F105" s="32" t="n">
-        <v>0.588</v>
+        <v>10.7</v>
       </c>
       <c r="G105" s="32" t="n">
-        <v>0.577</v>
-      </c>
-      <c r="H105" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
+        <v>10.4</v>
+      </c>
+      <c r="H105" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
         </is>
       </c>
       <c r="I105" s="32" t="inlineStr"/>
@@ -4462,37 +4738,37 @@
       </c>
       <c r="Q105" s="34" t="inlineStr">
         <is>
-          <t>Opp TS%</t>
+          <t>Opp BLK+STL</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
         <is>
-          <t>OREB%</t>
+          <t>TOV</t>
         </is>
       </c>
       <c r="B106" s="32" t="n">
-        <v>0.251</v>
+        <v>15.111</v>
       </c>
       <c r="C106" s="32" t="n">
-        <v>0.278</v>
+        <v>13.267</v>
       </c>
       <c r="D106" s="32" t="n">
-        <v>0.272</v>
+        <v>13.6</v>
       </c>
       <c r="E106" s="32" t="n">
-        <v>0.281</v>
+        <v>14.467</v>
       </c>
       <c r="F106" s="32" t="n">
-        <v>0.273</v>
+        <v>15.5</v>
       </c>
       <c r="G106" s="32" t="n">
-        <v>0.253</v>
-      </c>
-      <c r="H106" s="35" t="inlineStr">
-        <is>
-          <t>8th</t>
+        <v>15.4</v>
+      </c>
+      <c r="H106" s="33" t="inlineStr">
+        <is>
+          <t>12th</t>
         </is>
       </c>
       <c r="I106" s="32" t="inlineStr"/>
@@ -4532,282 +4808,6 @@
         </is>
       </c>
       <c r="Q106" s="34" t="inlineStr">
-        <is>
-          <t>Opp OREB%</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="31" t="inlineStr">
-        <is>
-          <t>REB</t>
-        </is>
-      </c>
-      <c r="B107" s="32" t="n">
-        <v>33</v>
-      </c>
-      <c r="C107" s="32" t="n">
-        <v>33.433</v>
-      </c>
-      <c r="D107" s="32" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="E107" s="32" t="n">
-        <v>33.933</v>
-      </c>
-      <c r="F107" s="32" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="G107" s="32" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="H107" s="35" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I107" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J107" s="35" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="K107" s="32" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="L107" s="32" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="M107" s="32" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="N107" s="32" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="O107" s="32" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="P107" s="32" t="n">
-        <v>34.889</v>
-      </c>
-      <c r="Q107" s="34" t="inlineStr">
-        <is>
-          <t>Opp REB</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="31" t="inlineStr">
-        <is>
-          <t>AST</t>
-        </is>
-      </c>
-      <c r="B108" s="32" t="n">
-        <v>22.556</v>
-      </c>
-      <c r="C108" s="32" t="n">
-        <v>20.567</v>
-      </c>
-      <c r="D108" s="32" t="n">
-        <v>20.45</v>
-      </c>
-      <c r="E108" s="32" t="n">
-        <v>20.733</v>
-      </c>
-      <c r="F108" s="32" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="G108" s="32" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="H108" s="35" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I108" s="32" t="inlineStr"/>
-      <c r="J108" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P108" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q108" s="34" t="inlineStr">
-        <is>
-          <t>Opp AST</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="31" t="inlineStr">
-        <is>
-          <t>BLK+STL</t>
-        </is>
-      </c>
-      <c r="B109" s="32" t="n">
-        <v>11.333</v>
-      </c>
-      <c r="C109" s="32" t="n">
-        <v>10</v>
-      </c>
-      <c r="D109" s="32" t="n">
-        <v>10.05</v>
-      </c>
-      <c r="E109" s="32" t="n">
-        <v>10.467</v>
-      </c>
-      <c r="F109" s="32" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="G109" s="32" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="H109" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I109" s="32" t="inlineStr"/>
-      <c r="J109" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P109" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q109" s="34" t="inlineStr">
-        <is>
-          <t>Opp BLK+STL</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="31" t="inlineStr">
-        <is>
-          <t>TOV</t>
-        </is>
-      </c>
-      <c r="B110" s="32" t="n">
-        <v>15.111</v>
-      </c>
-      <c r="C110" s="32" t="n">
-        <v>13.267</v>
-      </c>
-      <c r="D110" s="32" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="E110" s="32" t="n">
-        <v>14.467</v>
-      </c>
-      <c r="F110" s="32" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G110" s="32" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="H110" s="33" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I110" s="32" t="inlineStr"/>
-      <c r="J110" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P110" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q110" s="34" t="inlineStr">
         <is>
           <t>Opp TOV</t>
         </is>
@@ -4904,7 +4904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5044,17 +5044,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5934</v>
+        <v>0.6078</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-146</v>
+        <v>-155</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 59.3% (fair -146). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5180,13 +5180,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5704</v>
+        <v>0.5724</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-133</v>
+        <v>-134</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-113</v>
+        <v>-117</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5222,17 +5222,17 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Los Angeles Sparks @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -5242,17 +5242,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5359</v>
+        <v>0.5204</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-115</v>
+        <v>-109</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 52.0% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5312,13 +5312,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5402</v>
+        <v>0.5391</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>-117</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -5342,7 +5342,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5351,9 +5351,75 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.5425</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-119</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>-113</v>
+      </c>
+      <c r="I10" s="13">
+        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L10" s="18">
+        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M10" s="12">
+        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.2% (fair -119). Your call.</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="16">
+        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -5519,13 +5585,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4297</v>
+        <v>0.4291448</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>133</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -5549,7 +5615,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 43.0% (fair +133). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -5585,13 +5651,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5703</v>
+        <v>0.5708552</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-133</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-132</v>
+        <v>-126</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -5615,7 +5681,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -5647,17 +5713,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 10.5</t>
+          <t>Over 10</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4641</v>
+        <v>0.4514</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>-105</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -5681,7 +5747,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +115). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -5713,17 +5779,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Under 10</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5359</v>
+        <v>0.4667</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-115</v>
+        <v>114</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -5747,7 +5813,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -5783,13 +5849,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3831</v>
+        <v>0.3848</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -5813,7 +5879,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 38.5% (fair +160). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -5849,10 +5915,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6169</v>
+        <v>0.6152</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-161</v>
+        <v>-160</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-160</v>
@@ -5879,7 +5945,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 61.5% (fair -160). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6062,7 +6128,7 @@
         <v>146</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -6128,7 +6194,7 @@
         <v>-146</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -6184,17 +6250,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 172.5</t>
+          <t>Over 171</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5941506978584125</v>
+        <v>0.6279658307397271</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-146</v>
+        <v>-169</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -6218,7 +6284,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 62.8% (fair -169). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -6250,17 +6316,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 172.5</t>
+          <t>Under 171</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4058493021415875</v>
+        <v>0.3498341692602729</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -6284,7 +6350,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 35.0% (fair +186). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -6316,17 +6382,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky -5.5</t>
+          <t>Chicago Sky -3.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4228968214967185</v>
+        <v>0.4852393637430031</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -6350,7 +6416,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -6382,17 +6448,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm +5.5</t>
+          <t>Seattle Storm +3.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5771031785032815</v>
+        <v>0.5147606362569969</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-136</v>
+        <v>-106</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -6416,7 +6482,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -6458,7 +6524,7 @@
         <v>1157</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>567</v>
+        <v>545</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -6580,17 +6646,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 182.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5222822354138622</v>
+        <v>0.5204</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>-109</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -6614,7 +6680,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 52.0% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -6646,17 +6712,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 182.5</t>
+          <t>Under 181.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4777177645861378</v>
+        <v>0.4796</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>109</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -6680,7 +6746,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 48.0% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -6722,7 +6788,7 @@
         <v>109</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -6788,7 +6854,7 @@
         <v>-109</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -6848,13 +6914,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4553</v>
+        <v>0.4575</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -6878,7 +6944,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 45.8% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -6914,13 +6980,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5447</v>
+        <v>0.5425</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-120</v>
+        <v>-119</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -6944,7 +7010,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 54.2% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -7052,7 +7118,7 @@
         <v>141</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-105</v>
+        <v>-102</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -7118,7 +7184,7 @@
         <v>125</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -7184,7 +7250,7 @@
         <v>-111</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -7250,7 +7316,7 @@
         <v>220</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -7316,7 +7382,7 @@
         <v>-220</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -7372,17 +7438,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5934</v>
+        <v>0.6078</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-146</v>
+        <v>-155</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -7406,7 +7472,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 59.3% (fair -146). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -7438,17 +7504,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 165.5</t>
+          <t>Under 163.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4066</v>
+        <v>0.3922</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>100</v>
+        <v>-108</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -7472,7 +7538,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 40.7% (fair +146). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -7514,7 +7580,7 @@
         <v>-111</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-102</v>
+        <v>-105</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -7580,7 +7646,7 @@
         <v>111</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -7640,10 +7706,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4296</v>
+        <v>0.4276</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>122</v>
@@ -7670,7 +7736,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 43.0% (fair +133). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -7706,13 +7772,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5704</v>
+        <v>0.5724</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-133</v>
+        <v>-134</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-113</v>
+        <v>-117</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -7736,7 +7802,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -7772,13 +7838,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5402</v>
+        <v>0.5391</v>
       </c>
       <c r="G31" s="14" t="n">
         <v>-117</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -7802,7 +7868,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -7838,7 +7904,7 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4598</v>
+        <v>0.4609</v>
       </c>
       <c r="G32" s="14" t="n">
         <v>117</v>
@@ -7868,7 +7934,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -8381,7 +8447,7 @@
         <v>130</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>

</xml_diff>

<commit_message>
data: hourly update 2026-07-15 21:06Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-15.xlsx
+++ b/data/output/workbook/2026-07-15.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 15:21</t>
+          <t>2026-07-15 17:06</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1083,32 +1083,32 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>New York Mets +1.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6066</v>
+        <v>0.6346000000000001</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-154</v>
+        <v>-174</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -154). Your call.</t>
+          <t>Model 63.5% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1149,32 +1149,32 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings -1.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5367</v>
+        <v>0.6078</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-116</v>
+        <v>-155</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>104</v>
+        <v>-102</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1291,19 +1291,19 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Dallas Wings -1.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5319</v>
+        <v>0.5416</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-114</v>
+        <v>-118</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>-104</v>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1342,37 +1342,37 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>New York Liberty @ Dallas Wings</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Over 175.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5409</v>
+        <v>0.5368000000000001</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-118</v>
+        <v>-116</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 53.7% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -1405,9 +1405,75 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.5409</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I10" s="13">
+        <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF($H$10="","",$F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF($H$10="","",MAX(0,($F$10*IF($H$10&lt;0,-100/$H$10,$H$10/100)-(1-$F$10))/IF($H$10&lt;0,-100/$H$10,$H$10/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L10" s="18">
+        <f>IF($H$10="","",ROUND(MIN($K$10,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M10" s="12">
+        <f>IF($J$10="","",IF($J$10&lt;0,"Pass",IF($J$10&lt;'Settings'!$B$4,"Thin",IF($J$10&lt;0.06,"✅ Sharp band",IF($J$10&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>Model 54.1% (fair -118). Your call.</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="16">
+        <f>IF(OR($H$10="",$O$10=""),"",(1+IF($H$10&lt;0,-100/$H$10,$H$10/100))/(1+IF($O$10&lt;0,-100/$O$10,$O$10/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J9">
+  <conditionalFormatting sqref="J5:J10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1573,13 +1639,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4466</v>
+        <v>0.4481000000000001</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1603,7 +1669,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1639,10 +1705,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5534</v>
+        <v>0.5518999999999999</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-124</v>
+        <v>-123</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-124</v>
@@ -1669,7 +1735,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1705,13 +1771,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5161</v>
+        <v>0.5092</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-107</v>
+        <v>-104</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1735,7 +1801,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1771,13 +1837,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4839</v>
+        <v>0.4908</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -1801,7 +1867,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1837,13 +1903,13 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3755</v>
+        <v>0.3654</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1867,7 +1933,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 37.5% (fair +166). Your call.</t>
+          <t>Model 36.5% (fair +174). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -1903,13 +1969,13 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6245000000000001</v>
+        <v>0.6346000000000001</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-166</v>
+        <v>-174</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-175</v>
+        <v>160</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -1933,7 +1999,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.5% (fair -166). Your call.</t>
+          <t>Model 63.5% (fair -174). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2238,14 +2304,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 167.5</t>
+          <t>Over 167</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5850016819596556</v>
+        <v>0.5964301472202969</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-141</v>
+        <v>-148</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>113</v>
@@ -2272,7 +2338,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 58.5% (fair -141). Your call.</t>
+          <t>Model 59.6% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2304,17 +2370,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 167.5</t>
+          <t>Under 167</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4149983180403444</v>
+        <v>0.3807698527797032</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-101</v>
+        <v>113</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2338,7 +2404,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 41.5% (fair +141). Your call.</t>
+          <t>Model 38.1% (fair +163). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2512,7 +2578,7 @@
         <v>220</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -2638,13 +2704,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6066</v>
+        <v>0.6078</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-154</v>
+        <v>-155</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -2668,7 +2734,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -154). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2704,10 +2770,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3934</v>
+        <v>0.3922</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>-108</v>
@@ -2734,7 +2800,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 39.3% (fair +154). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2766,17 +2832,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics -5.5</t>
+          <t>Washington Mystics -6.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5118</v>
+        <v>0.4956023001506284</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-105</v>
+        <v>102</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-105</v>
+        <v>113</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2800,7 +2866,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -2832,17 +2898,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +5.5</t>
+          <t>Portland Fire +6.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4882</v>
+        <v>0.5043976998493716</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>105</v>
+        <v>-102</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-108</v>
+        <v>104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2866,7 +2932,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -3034,10 +3100,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5319</v>
+        <v>0.5368000000000001</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-114</v>
+        <v>-116</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>-104</v>
@@ -3064,7 +3130,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 53.7% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -3100,13 +3166,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4681</v>
+        <v>0.4631999999999999</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -3130,7 +3196,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 46.3% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -3166,13 +3232,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5367</v>
+        <v>0.5416</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-116</v>
+        <v>-118</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -3196,7 +3262,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -3232,10 +3298,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4633</v>
+        <v>0.4584</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>100</v>
@@ -3262,7 +3328,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-15 23:04Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-15.xlsx
+++ b/data/output/workbook/2026-07-15.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 17:06</t>
+          <t>2026-07-15 19:04</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1108,7 +1108,7 @@
         <v>-174</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6078</v>
+        <v>0.6101</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-155</v>
+        <v>-156</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-102</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 61.0% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1234,13 +1234,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5693</v>
+        <v>0.5686</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>-132</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1408,37 +1408,37 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Indiana Fever</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5409</v>
+        <v>0.5028</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-118</v>
+        <v>-101</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-110</v>
+        <v>104</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -1471,9 +1471,75 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Portland Fire @ Washington Mystics</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Washington Mystics -6.5</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>0.4905</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>104</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="I11" s="13">
+        <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>IF($H$11="","",$F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IF($H$11="","",MAX(0,($F$11*IF($H$11&lt;0,-100/$H$11,$H$11/100)-(1-$F$11))/IF($H$11&lt;0,-100/$H$11,$H$11/100))*'Settings'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="L11" s="18">
+        <f>IF($H$11="","",ROUND(MIN($K$11,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
+        <v/>
+      </c>
+      <c r="M11" s="12">
+        <f>IF($J$11="","",IF($J$11&lt;0,"Pass",IF($J$11&lt;'Settings'!$B$4,"Thin",IF($J$11&lt;0.06,"✅ Sharp band",IF($J$11&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
+        <v/>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>Model 49.0% (fair +104). Your call.</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="16">
+        <f>IF(OR($H$11="",$O$11=""),"",(1+IF($H$11&lt;0,-100/$H$11,$H$11/100))/(1+IF($O$11&lt;0,-100/$O$11,$O$11/100))-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J10">
+  <conditionalFormatting sqref="J5:J11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -1639,13 +1705,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4481000000000001</v>
+        <v>0.4488</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>123</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -1669,7 +1735,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -1705,7 +1771,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5518999999999999</v>
+        <v>0.5512</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-123</v>
@@ -1735,7 +1801,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -1771,13 +1837,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5092</v>
+        <v>0.5028</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-104</v>
+        <v>-101</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -1801,7 +1867,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -1837,10 +1903,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4908</v>
+        <v>0.4972</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>100</v>
@@ -1867,7 +1933,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -1909,7 +1975,7 @@
         <v>174</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -1975,7 +2041,7 @@
         <v>-174</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -2176,13 +2242,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4591</v>
+        <v>0.445452</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>113</v>
+        <v>150</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -2206,7 +2272,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 44.5% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -2242,13 +2308,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5409</v>
+        <v>0.554548</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-118</v>
+        <v>-124</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-110</v>
+        <v>-120</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -2272,7 +2338,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 55.5% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -2304,17 +2370,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 167</t>
+          <t>Over 167.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5964301472202969</v>
+        <v>0.5850016819596556</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-148</v>
+        <v>-141</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -2338,7 +2404,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 59.6% (fair -148). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -2370,17 +2436,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 167</t>
+          <t>Under 167.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3807698527797032</v>
+        <v>0.4149983180403444</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -2404,7 +2470,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 38.1% (fair +163). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -2436,17 +2502,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -2.5</t>
+          <t>Indiana Fever -3.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4595470900789442</v>
+        <v>0.4284526556424175</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -2470,7 +2536,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +118). Your call.</t>
+          <t>Model 42.8% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -2502,14 +2568,14 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +2.5</t>
+          <t>Golden State Valkyries +3.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5404529099210558</v>
+        <v>0.5715473443575825</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-118</v>
+        <v>-133</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>117</v>
@@ -2536,7 +2602,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -118). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -2704,10 +2770,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.6078</v>
+        <v>0.6101</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-155</v>
+        <v>-156</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>-102</v>
@@ -2734,7 +2800,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 61.0% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -2770,13 +2836,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.3922</v>
+        <v>0.3899</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -2800,7 +2866,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 39.2% (fair +155). Your call.</t>
+          <t>Model 39.0% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -2836,13 +2902,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4956023001506284</v>
+        <v>0.4905</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -2866,7 +2932,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -2902,13 +2968,13 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5043976998493716</v>
+        <v>0.5095000000000001</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -2932,7 +2998,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -2968,13 +3034,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4307</v>
+        <v>0.4314</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>132</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -3034,13 +3100,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5693</v>
+        <v>0.5686</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>-132</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-113</v>
+        <v>-115</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -3709,7 +3775,7 @@
         <v>130</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>

</xml_diff>